<commit_message>
APROJ File Processing by FullLeg
- FullLeg: object will now accept .aproj file input as opposed to .asim only
- FullLeg:optimize_forces: modified bounds to avoid Am saturation
- legScaler: now dynamically changes floor height to accommodate new leg size
- paramChanger: allows user to change all VE properties of an input file to determine how scaling impacts performance
- processSimData: will now determine whether jsystem is on the path and if not, add it
- ParameterCalculation/LRSolver: now allows users to set LR parameters based on min-max scheme or neutral position scheme
- Canvas/CanvasModel:create_animatlab_project: now dynamically determines JointMotion and PassiveTension output datatool names
</commit_message>
<xml_diff>
--- a/ParameterCalculation/MuscleParameters_20190513.xlsx
+++ b/ParameterCalculation/MuscleParameters_20190513.xlsx
@@ -669,19 +669,19 @@
         <v>12.210800000000003</v>
       </c>
       <c r="G2">
-        <v>1190.29</v>
+        <v>283.411</v>
       </c>
       <c r="H2">
-        <v>379.39</v>
+        <v>3601.22</v>
       </c>
       <c r="I2">
-        <v>16.101784271059994</v>
+        <v>1673.5886930994211</v>
       </c>
       <c r="J2">
         <v>459.5</v>
       </c>
       <c r="K2">
-        <v>-161.03694886263483</v>
+        <v>-16.735886930994212</v>
       </c>
       <c r="L2">
         <v>-60</v>
@@ -693,19 +693,19 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>16.101784271059994</v>
+        <v>1673.5886930994211</v>
       </c>
       <c r="P2">
-        <v>1.6026400000000001</v>
+        <v>1.0803750000000232</v>
       </c>
       <c r="Q2">
-        <v>2.5731200000000003</v>
+        <v>2.1607500000000464</v>
       </c>
       <c r="R2">
-        <v>3.5436000000000001</v>
+        <v>3.2411250000000695</v>
       </c>
       <c r="S2">
-        <v>1.7718459586920456</v>
+        <v>1.9724858602155215</v>
       </c>
       <c r="T2">
         <v>12.21</v>
@@ -737,19 +737,19 @@
         <v>1.0388000000000002</v>
       </c>
       <c r="G3">
-        <v>8924.08</v>
+        <v>208.91399999999999</v>
       </c>
       <c r="H3">
-        <v>5189.3</v>
+        <v>4676.34</v>
       </c>
       <c r="I3">
-        <v>1.6447538793914893</v>
+        <v>243.19404922599733</v>
       </c>
       <c r="J3">
         <v>459.5</v>
       </c>
       <c r="K3">
-        <v>-16.449490435866533</v>
+        <v>-2.4319404922599732</v>
       </c>
       <c r="L3">
         <v>-60</v>
@@ -761,19 +761,19 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>1.6447538793914893</v>
+        <v>243.19404922599733</v>
       </c>
       <c r="P3">
-        <v>1.36154</v>
+        <v>0.7732899999999896</v>
       </c>
       <c r="Q3">
-        <v>1.9429950000000002</v>
+        <v>1.5465799999999792</v>
       </c>
       <c r="R3">
-        <v>2.5244499999999999</v>
+        <v>2.3198699999999688</v>
       </c>
       <c r="S3">
-        <v>1.0615867322472212</v>
+        <v>1.4118279216438805</v>
       </c>
       <c r="T3">
         <v>1.04</v>
@@ -805,19 +805,19 @@
         <v>3.0184000000000006</v>
       </c>
       <c r="G4">
-        <v>47.45</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>3663.78</v>
+        <v>1091.0899999999999</v>
       </c>
       <c r="I4">
-        <v>236.20473340358271</v>
+        <v>32981.118000000002</v>
       </c>
       <c r="J4">
         <v>459.5</v>
       </c>
       <c r="K4">
-        <v>-2362.3276112691942</v>
+        <v>-329.81118000000004</v>
       </c>
       <c r="L4">
         <v>-60</v>
@@ -829,19 +829,19 @@
         <v>0</v>
       </c>
       <c r="O4">
-        <v>236.20473340358271</v>
+        <v>32981.118000000002</v>
       </c>
       <c r="P4">
-        <v>2.2126700000000001</v>
+        <v>1.4095599999999717</v>
       </c>
       <c r="Q4">
-        <v>4.0161449999999999</v>
+        <v>2.8191199999999434</v>
       </c>
       <c r="R4">
-        <v>5.8196199999999996</v>
+        <v>4.2286799999999154</v>
       </c>
       <c r="S4">
-        <v>3.2926797979887645</v>
+        <v>2.5734926938565548</v>
       </c>
       <c r="T4">
         <v>3.02</v>
@@ -873,19 +873,19 @@
         <v>3.3908000000000005</v>
       </c>
       <c r="G5">
-        <v>47.45</v>
+        <v>6.5278999999999998</v>
       </c>
       <c r="H5">
-        <v>1081.52</v>
+        <v>1474.59</v>
       </c>
       <c r="I5">
-        <v>237.92834562697576</v>
+        <v>22689.040886042985</v>
       </c>
       <c r="J5">
         <v>459.5</v>
       </c>
       <c r="K5">
-        <v>-2379.565778717285</v>
+        <v>-226.89040886042986</v>
       </c>
       <c r="L5">
         <v>-60</v>
@@ -897,19 +897,19 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>237.92834562697576</v>
+        <v>22689.040886042985</v>
       </c>
       <c r="P5">
-        <v>2.9523299999999999</v>
+        <v>2.2569099999999587</v>
       </c>
       <c r="Q5">
-        <v>4.8046499999999996</v>
+        <v>4.5138199999999173</v>
       </c>
       <c r="R5">
-        <v>6.6569699999999994</v>
+        <v>6.770729999999876</v>
       </c>
       <c r="S5">
-        <v>3.3818581590598966</v>
+        <v>4.1205350575298727</v>
       </c>
       <c r="T5">
         <v>10</v>
@@ -941,19 +941,19 @@
         <v>12.485200000000003</v>
       </c>
       <c r="G6">
-        <v>29.35</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>373.96</v>
+        <v>1469.09</v>
       </c>
       <c r="I6">
-        <v>171.63004770017037</v>
+        <v>91869.570500000002</v>
       </c>
       <c r="J6">
         <v>459.5</v>
       </c>
       <c r="K6">
-        <v>-1716.504130816083</v>
+        <v>-918.69570500000009</v>
       </c>
       <c r="L6">
         <v>-60</v>
@@ -965,19 +965,19 @@
         <v>0</v>
       </c>
       <c r="O6">
-        <v>171.63004770017037</v>
+        <v>91869.570500000002</v>
       </c>
       <c r="P6">
-        <v>2.3701400000000001</v>
+        <v>2.1288699999999765</v>
       </c>
       <c r="Q6">
-        <v>4.5753550000000001</v>
+        <v>4.257739999999953</v>
       </c>
       <c r="R6">
-        <v>6.78057</v>
+        <v>6.3866099999999291</v>
       </c>
       <c r="S6">
-        <v>4.026153332162516</v>
+        <v>3.8867670699866999</v>
       </c>
       <c r="T6">
         <v>12.49</v>
@@ -1009,19 +1009,19 @@
         <v>2.0580000000000003</v>
       </c>
       <c r="G7">
-        <v>685.43</v>
+        <v>207.77199999999999</v>
       </c>
       <c r="H7">
-        <v>9080.2000000000007</v>
+        <v>3512.26</v>
       </c>
       <c r="I7">
-        <v>29.349748041375491</v>
+        <v>368.83054117012881</v>
       </c>
       <c r="J7">
         <v>459.5</v>
       </c>
       <c r="K7">
-        <v>-293.53230641432879</v>
+        <v>-3.6883054117012883</v>
       </c>
       <c r="L7">
         <v>-60</v>
@@ -1033,19 +1033,19 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>29.349748041375491</v>
+        <v>368.83054117012881</v>
       </c>
       <c r="P7">
-        <v>3.6246</v>
+        <v>2.1263000000000098</v>
       </c>
       <c r="Q7">
-        <v>4.1267849999999999</v>
+        <v>4.2526000000000197</v>
       </c>
       <c r="R7">
-        <v>4.6289700000000007</v>
+        <v>6.3789000000000291</v>
       </c>
       <c r="S7">
-        <v>0.916860175135773</v>
+        <v>3.8820749134107997</v>
       </c>
       <c r="T7">
         <v>2.06</v>
@@ -1077,19 +1077,19 @@
         <v>2.21</v>
       </c>
       <c r="G8">
-        <v>1545.95</v>
+        <v>1891.33</v>
       </c>
       <c r="H8">
-        <v>81.900000000000006</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>2.3270794657007019</v>
+        <v>22.111684898986429</v>
       </c>
       <c r="J8">
         <v>459.5</v>
       </c>
       <c r="K8">
-        <v>-23.273555936957148</v>
+        <v>-0.22111684898986428</v>
       </c>
       <c r="L8">
         <v>-60</v>
@@ -1101,19 +1101,19 @@
         <v>0</v>
       </c>
       <c r="O8">
-        <v>2.3270794657007019</v>
+        <v>22.111684898986429</v>
       </c>
       <c r="P8">
-        <v>6.0133799999999997</v>
+        <v>3.3155900000000189</v>
       </c>
       <c r="Q8">
-        <v>6.5287550000000003</v>
+        <v>6.6311800000000378</v>
       </c>
       <c r="R8">
-        <v>7.04413</v>
+        <v>9.9467700000000576</v>
       </c>
       <c r="S8">
-        <v>0.94094171024741624</v>
+        <v>6.0534114481285464</v>
       </c>
       <c r="T8">
         <v>2.21</v>
@@ -1145,19 +1145,19 @@
         <v>11.015200000000002</v>
       </c>
       <c r="G9">
-        <v>105.51</v>
+        <v>788.74400000000003</v>
       </c>
       <c r="H9">
-        <v>7235.72</v>
+        <v>722.25599999999997</v>
       </c>
       <c r="I9">
-        <v>766.75532745711303</v>
+        <v>211.11057580152746</v>
       </c>
       <c r="J9">
         <v>459.5</v>
       </c>
       <c r="K9">
-        <v>-7668.4630957197278</v>
+        <v>-2.1111057580152748</v>
       </c>
       <c r="L9">
         <v>-60</v>
@@ -1169,19 +1169,19 @@
         <v>0</v>
       </c>
       <c r="O9">
-        <v>766.75532745711303</v>
+        <v>211.11057580152746</v>
       </c>
       <c r="P9">
-        <v>5.75875</v>
+        <v>3.2996399999999335</v>
       </c>
       <c r="Q9">
-        <v>6.0958699999999997</v>
+        <v>6.599279999999867</v>
       </c>
       <c r="R9">
-        <v>6.4329899999999993</v>
+        <v>9.8989199999997997</v>
       </c>
       <c r="S9">
-        <v>0.61549409528713817</v>
+        <v>6.024290865487699</v>
       </c>
       <c r="T9">
         <v>11.02</v>
@@ -1213,19 +1213,19 @@
         <v>0.44100000000000006</v>
       </c>
       <c r="G10">
-        <v>14.6</v>
+        <v>1096</v>
       </c>
       <c r="H10">
-        <v>9987.7199999999993</v>
+        <v>510.11399999999998</v>
       </c>
       <c r="I10">
-        <v>301.43978082191785</v>
+        <v>6.4479029197080289</v>
       </c>
       <c r="J10">
         <v>459.5</v>
       </c>
       <c r="K10">
-        <v>-3014.7554924475098</v>
+        <v>-6.447902919708029E-2</v>
       </c>
       <c r="L10">
         <v>-60</v>
@@ -1237,19 +1237,19 @@
         <v>0</v>
       </c>
       <c r="O10">
-        <v>301.43978082191785</v>
+        <v>6.4479029197080289</v>
       </c>
       <c r="P10">
-        <v>5.6810899999999993</v>
+        <v>3.1614650000000708</v>
       </c>
       <c r="Q10">
-        <v>5.9755200000000004</v>
+        <v>6.3229300000001416</v>
       </c>
       <c r="R10">
-        <v>6.2699500000000006</v>
+        <v>9.4843950000002124</v>
       </c>
       <c r="S10">
-        <v>0.53755317535415414</v>
+        <v>5.7720189842103622</v>
       </c>
       <c r="T10">
         <v>0.44</v>
@@ -1281,19 +1281,19 @@
         <v>2.8518000000000003</v>
       </c>
       <c r="G11">
-        <v>6249.83</v>
+        <v>364.702</v>
       </c>
       <c r="H11">
-        <v>288.45</v>
+        <v>3025.12</v>
       </c>
       <c r="I11">
-        <v>2.9815367778003563</v>
+        <v>264.9010068494278</v>
       </c>
       <c r="J11">
         <v>459.5</v>
       </c>
       <c r="K11">
-        <v>-29.818905627847737</v>
+        <v>-2.6490100684942779</v>
       </c>
       <c r="L11">
         <v>-60</v>
@@ -1305,19 +1305,19 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>2.9815367778003563</v>
+        <v>264.9010068494278</v>
       </c>
       <c r="P11">
-        <v>1.42676</v>
+        <v>0.71427499999999189</v>
       </c>
       <c r="Q11">
-        <v>1.499795</v>
+        <v>1.4285499999999838</v>
       </c>
       <c r="R11">
-        <v>1.5728300000000002</v>
+        <v>2.1428249999999758</v>
       </c>
       <c r="S11">
-        <v>0.13334305662463272</v>
+        <v>1.3040817658733268</v>
       </c>
       <c r="T11">
         <v>2.85</v>
@@ -1349,19 +1349,19 @@
         <v>0.37240000000000006</v>
       </c>
       <c r="G12">
-        <v>20.3</v>
+        <v>92.297899999999998</v>
       </c>
       <c r="H12">
-        <v>122.89</v>
+        <v>324.81099999999998</v>
       </c>
       <c r="I12">
-        <v>35.268472906403943</v>
+        <v>225.95795787336439</v>
       </c>
       <c r="J12">
         <v>459.5</v>
       </c>
       <c r="K12">
-        <v>-352.72657814076564</v>
+        <v>-2.2595795787336441</v>
       </c>
       <c r="L12">
         <v>-60</v>
@@ -1373,19 +1373,19 @@
         <v>0</v>
       </c>
       <c r="O12">
-        <v>35.268472906403943</v>
+        <v>225.95795787336439</v>
       </c>
       <c r="P12">
-        <v>0.94296199999999997</v>
+        <v>0.61124499999999005</v>
       </c>
       <c r="Q12">
-        <v>1.3181259999999999</v>
+        <v>1.2224899999999801</v>
       </c>
       <c r="R12">
-        <v>1.6932900000000002</v>
+        <v>1.8337349999999701</v>
       </c>
       <c r="S12">
-        <v>0.68495261854622724</v>
+        <v>1.115975582207466</v>
       </c>
       <c r="T12">
         <v>5</v>
@@ -1417,19 +1417,19 @@
         <v>9.231600000000002</v>
       </c>
       <c r="G13">
-        <v>2127.83</v>
+        <v>7.7950999999999997</v>
       </c>
       <c r="H13">
-        <v>19.62</v>
+        <v>1646.01</v>
       </c>
       <c r="I13">
-        <v>9.3151067049529335</v>
+        <v>19582.328736000825</v>
       </c>
       <c r="J13">
         <v>459.5</v>
       </c>
       <c r="K13">
-        <v>-93.162120224875011</v>
+        <v>-195.82328736000827</v>
       </c>
       <c r="L13">
         <v>-60</v>
@@ -1441,19 +1441,19 @@
         <v>0</v>
       </c>
       <c r="O13">
-        <v>9.3151067049529335</v>
+        <v>19582.328736000825</v>
       </c>
       <c r="P13">
-        <v>1.47803</v>
+        <v>0.96281999999999046</v>
       </c>
       <c r="Q13">
-        <v>1.8418499999999998</v>
+        <v>1.9256399999999809</v>
       </c>
       <c r="R13">
-        <v>2.20567</v>
+        <v>2.8884599999999714</v>
       </c>
       <c r="S13">
-        <v>0.66424140290509825</v>
+        <v>1.7578607760570626</v>
       </c>
       <c r="T13">
         <v>9.23</v>
@@ -1485,19 +1485,19 @@
         <v>18.737600000000004</v>
       </c>
       <c r="G14">
-        <v>7684.17</v>
+        <v>394.77199999999999</v>
       </c>
       <c r="H14">
-        <v>441.28</v>
+        <v>3466.41</v>
       </c>
       <c r="I14">
-        <v>19.8161848319337</v>
+        <v>1832.9200318158328</v>
       </c>
       <c r="J14">
         <v>459.5</v>
       </c>
       <c r="K14">
-        <v>-198.18536192713211</v>
+        <v>-18.329200318158328</v>
       </c>
       <c r="L14">
         <v>-60</v>
@@ -1509,19 +1509,19 @@
         <v>0</v>
       </c>
       <c r="O14">
-        <v>19.8161848319337</v>
+        <v>1832.9200318158328</v>
       </c>
       <c r="P14">
-        <v>2.1087199999999999</v>
+        <v>1.0981799999999848</v>
       </c>
       <c r="Q14">
-        <v>2.5653700000000002</v>
+        <v>2.1963599999999697</v>
       </c>
       <c r="R14">
-        <v>3.0220199999999999</v>
+        <v>3.2945399999999547</v>
       </c>
       <c r="S14">
-        <v>0.83372501961578005</v>
+        <v>2.0049931940033834</v>
       </c>
       <c r="T14">
         <v>18.739999999999998</v>
@@ -1553,19 +1553,19 @@
         <v>7.3892000000000007</v>
       </c>
       <c r="G15">
-        <v>52.16</v>
+        <v>1208.8599999999999</v>
       </c>
       <c r="H15">
-        <v>8512.42</v>
+        <v>4703.34</v>
       </c>
       <c r="I15">
-        <v>1213.4249654907974</v>
+        <v>361.42446602584255</v>
       </c>
       <c r="J15">
         <v>459.5</v>
       </c>
       <c r="K15">
-        <v>-12135.689488002452</v>
+        <v>-3.6142446602584255</v>
       </c>
       <c r="L15">
         <v>-60</v>
@@ -1577,19 +1577,19 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>1213.4249654907974</v>
+        <v>361.42446602584255</v>
       </c>
       <c r="P15">
-        <v>1.96549</v>
+        <v>1.0033999999999903</v>
       </c>
       <c r="Q15">
-        <v>2.333275</v>
+        <v>2.0067999999999806</v>
       </c>
       <c r="R15">
-        <v>2.70106</v>
+        <v>3.0101999999999705</v>
       </c>
       <c r="S15">
-        <v>0.67148046937345829</v>
+        <v>1.8319493806689278</v>
       </c>
       <c r="T15">
         <v>7.39</v>
@@ -1621,19 +1621,19 @@
         <v>1.5484000000000002</v>
       </c>
       <c r="G16">
-        <v>516.08000000000004</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>689.56</v>
+        <v>1188.95</v>
       </c>
       <c r="I16">
-        <v>3.6210316230041846</v>
+        <v>9229.8625000000011</v>
       </c>
       <c r="J16">
         <v>459.5</v>
       </c>
       <c r="K16">
-        <v>-36.214612895526095</v>
+        <v>-92.298625000000015</v>
       </c>
       <c r="L16">
         <v>-60</v>
@@ -1645,19 +1645,19 @@
         <v>0</v>
       </c>
       <c r="O16">
-        <v>3.6210316230041846</v>
+        <v>9229.8625000000011</v>
       </c>
       <c r="P16">
-        <v>2.1859900000000003</v>
+        <v>1.4393300000000049</v>
       </c>
       <c r="Q16">
-        <v>4.1566049999999999</v>
+        <v>2.8786600000000098</v>
       </c>
       <c r="R16">
-        <v>6.1272199999999994</v>
+        <v>4.3179900000000142</v>
       </c>
       <c r="S16">
-        <v>3.5978342921934763</v>
+        <v>2.6278450289797117</v>
       </c>
       <c r="T16">
         <v>1.55</v>
@@ -1689,19 +1689,19 @@
         <v>2.3520000000000003</v>
       </c>
       <c r="G17">
-        <v>47.45</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>3327.05</v>
+        <v>1456.59</v>
       </c>
       <c r="I17">
-        <v>167.1248682824025</v>
+        <v>17138.432499999999</v>
       </c>
       <c r="J17">
         <v>459.5</v>
       </c>
       <c r="K17">
-        <v>-1671.4469908555116</v>
+        <v>-171.38432499999999</v>
       </c>
       <c r="L17">
         <v>-60</v>
@@ -1713,19 +1713,19 @@
         <v>0</v>
       </c>
       <c r="O17">
-        <v>167.1248682824025</v>
+        <v>17138.432499999999</v>
       </c>
       <c r="P17">
-        <v>2.0736300000000001</v>
+        <v>1.6045399999999792</v>
       </c>
       <c r="Q17">
-        <v>4.1628049999999996</v>
+        <v>3.2090799999999584</v>
       </c>
       <c r="R17">
-        <v>6.2519799999999996</v>
+        <v>4.8136199999999381</v>
       </c>
       <c r="S17">
-        <v>3.814294246919518</v>
+        <v>2.9294758413977595</v>
       </c>
       <c r="T17">
         <v>2.35</v>
@@ -1757,19 +1757,19 @@
         <v>11.279800000000002</v>
       </c>
       <c r="G18">
-        <v>20.3</v>
+        <v>64.297899999999998</v>
       </c>
       <c r="H18">
-        <v>275.36</v>
+        <v>163.864</v>
       </c>
       <c r="I18">
-        <v>164.28792118226599</v>
+        <v>400.27220671281646</v>
       </c>
       <c r="J18">
         <v>459.5</v>
       </c>
       <c r="K18">
-        <v>-1643.0741535723919</v>
+        <v>-4.0027220671281647</v>
       </c>
       <c r="L18">
         <v>-60</v>
@@ -1781,19 +1781,19 @@
         <v>0</v>
       </c>
       <c r="O18">
-        <v>164.28792118226599</v>
+        <v>400.27220671281646</v>
       </c>
       <c r="P18">
-        <v>2.1748400000000001</v>
+        <v>1.2457200000000048</v>
       </c>
       <c r="Q18">
-        <v>2.5796900000000003</v>
+        <v>2.4914400000000096</v>
       </c>
       <c r="R18">
-        <v>2.98454</v>
+        <v>3.7371600000000145</v>
       </c>
       <c r="S18">
-        <v>0.73915159135322162</v>
+        <v>2.2743631477844604</v>
       </c>
       <c r="T18">
         <v>11.28</v>
@@ -1825,19 +1825,19 @@
         <v>18.257400000000004</v>
       </c>
       <c r="G19">
-        <v>425.51</v>
+        <v>149.005</v>
       </c>
       <c r="H19">
-        <v>9979.59</v>
+        <v>421.25599999999997</v>
       </c>
       <c r="I19">
-        <v>446.5162416864469</v>
+        <v>698.83331834502201</v>
       </c>
       <c r="J19">
         <v>459.5</v>
       </c>
       <c r="K19">
-        <v>-4465.6922467923887</v>
+        <v>-6.9883331834502203</v>
       </c>
       <c r="L19">
         <v>-60</v>
@@ -1849,19 +1849,19 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <v>446.5162416864469</v>
+        <v>698.83331834502201</v>
       </c>
       <c r="P19">
-        <v>4.9908000000000001</v>
+        <v>2.6223899945745761</v>
       </c>
       <c r="Q19">
-        <v>5.1396649999999999</v>
+        <v>5.2447799891491522</v>
       </c>
       <c r="R19">
-        <v>5.2885300000000006</v>
+        <v>7.8671699837237288</v>
       </c>
       <c r="S19">
-        <v>0.27178906174335538</v>
+        <v>4.7878071820144852</v>
       </c>
       <c r="T19">
         <v>18.260000000000002</v>
@@ -1893,19 +1893,19 @@
         <v>11.642400000000002</v>
       </c>
       <c r="G20">
-        <v>813.07</v>
+        <v>67.004800000000003</v>
       </c>
       <c r="H20">
-        <v>4745.25</v>
+        <v>1841.26</v>
       </c>
       <c r="I20">
-        <v>79.573523558857175</v>
+        <v>3315.0165767228618</v>
       </c>
       <c r="J20">
         <v>459.5</v>
       </c>
       <c r="K20">
-        <v>-795.82965641880241</v>
+        <v>-33.150165767228621</v>
       </c>
       <c r="L20">
         <v>-60</v>
@@ -1917,19 +1917,19 @@
         <v>0</v>
       </c>
       <c r="O20">
-        <v>79.573523558857175</v>
+        <v>3315.0165767228618</v>
       </c>
       <c r="P20">
-        <v>4.68886</v>
+        <v>2.5105450000000507</v>
       </c>
       <c r="Q20">
-        <v>5.0254599999999998</v>
+        <v>5.0210900000001013</v>
       </c>
       <c r="R20">
-        <v>5.3620599999999996</v>
+        <v>7.5316350000001533</v>
       </c>
       <c r="S20">
-        <v>0.61454470952079587</v>
+        <v>4.5836070937727831</v>
       </c>
       <c r="T20">
         <v>11.64</v>
@@ -1961,19 +1961,19 @@
         <v>7.1736000000000013</v>
       </c>
       <c r="G21">
-        <v>5229.6099999999997</v>
+        <v>1292.77</v>
       </c>
       <c r="H21">
-        <v>6281.77</v>
+        <v>3319.34</v>
       </c>
       <c r="I21">
-        <v>15.782552542158976</v>
+        <v>255.79823711874505</v>
       </c>
       <c r="J21">
         <v>459.5</v>
       </c>
       <c r="K21">
-        <v>-157.84425277771956</v>
+        <v>-2.5579823711874505</v>
       </c>
       <c r="L21">
         <v>-60</v>
@@ -1985,19 +1985,19 @@
         <v>0</v>
       </c>
       <c r="O21">
-        <v>15.782552542158976</v>
+        <v>255.79823711874505</v>
       </c>
       <c r="P21">
-        <v>1.10378</v>
+        <v>0.55407000000000473</v>
       </c>
       <c r="Q21">
-        <v>1.1771850000000001</v>
+        <v>1.1081400000000095</v>
       </c>
       <c r="R21">
-        <v>1.2505900000000001</v>
+        <v>1.662210000000014</v>
       </c>
       <c r="S21">
-        <v>0.1340185811122224</v>
+        <v>1.0115887914562998</v>
       </c>
       <c r="T21">
         <v>7.17</v>
@@ -2029,19 +2029,19 @@
         <v>3.0086000000000004</v>
       </c>
       <c r="G22">
-        <v>1.18</v>
+        <v>845.77200000000005</v>
       </c>
       <c r="H22">
-        <v>9980.6299999999992</v>
+        <v>2482.9</v>
       </c>
       <c r="I22">
-        <v>25462.074661016948</v>
+        <v>118.46340053820651</v>
       </c>
       <c r="J22">
         <v>459.5</v>
       </c>
       <c r="K22">
-        <v>-254650.9595518788</v>
+        <v>-1.1846340053820652</v>
       </c>
       <c r="L22">
         <v>-60</v>
@@ -2053,19 +2053,19 @@
         <v>0</v>
       </c>
       <c r="O22">
-        <v>25462.074661016948</v>
+        <v>118.46340053820651</v>
       </c>
       <c r="P22">
-        <v>1.3892200000000001</v>
+        <v>0.78364000000001777</v>
       </c>
       <c r="Q22">
-        <v>1.5067900000000001</v>
+        <v>1.5672800000000355</v>
       </c>
       <c r="R22">
-        <v>1.62436</v>
+        <v>2.3509200000000532</v>
       </c>
       <c r="S22">
-        <v>0.21465247028627457</v>
+        <v>1.4307243498778603</v>
       </c>
       <c r="T22">
         <v>3.01</v>
@@ -2097,19 +2097,19 @@
         <v>4.9294000000000011</v>
       </c>
       <c r="G23">
-        <v>2822.38</v>
+        <v>196.77199999999999</v>
       </c>
       <c r="H23">
-        <v>8369.92</v>
+        <v>3040.97</v>
       </c>
       <c r="I23">
-        <v>19.55018069855937</v>
+        <v>811.19610818612398</v>
       </c>
       <c r="J23">
         <v>459.5</v>
       </c>
       <c r="K23">
-        <v>-195.52500495660416</v>
+        <v>-8.1119610818612404</v>
       </c>
       <c r="L23">
         <v>-60</v>
@@ -2121,19 +2121,19 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>19.55018069855937</v>
+        <v>811.19610818612398</v>
       </c>
       <c r="P23">
-        <v>1.7914400000000001</v>
+        <v>1.0917450000000231</v>
       </c>
       <c r="Q23">
-        <v>2.4638849999999999</v>
+        <v>2.1834900000000461</v>
       </c>
       <c r="R23">
-        <v>3.1363299999999996</v>
+        <v>3.2752350000000692</v>
       </c>
       <c r="S23">
-        <v>1.2277109839385376</v>
+        <v>1.9932445451449672</v>
       </c>
       <c r="T23">
         <v>4.93</v>
@@ -2165,19 +2165,19 @@
         <v>3.9592000000000005</v>
       </c>
       <c r="G24">
-        <v>23.31</v>
+        <v>722.78399999999999</v>
       </c>
       <c r="H24">
-        <v>9608.56</v>
+        <v>781.31100000000004</v>
       </c>
       <c r="I24">
-        <v>1636.3022393822393</v>
+        <v>82.406586200026567</v>
       </c>
       <c r="J24">
         <v>459.5</v>
       </c>
       <c r="K24">
-        <v>-16364.964007176195</v>
+        <v>-0.82406586200026566</v>
       </c>
       <c r="L24">
         <v>-60</v>
@@ -2189,19 +2189,19 @@
         <v>0</v>
       </c>
       <c r="O24">
-        <v>1636.3022393822393</v>
+        <v>82.406586200026567</v>
       </c>
       <c r="P24">
-        <v>4.8204700000000003</v>
+        <v>2.6490000711022086</v>
       </c>
       <c r="Q24">
-        <v>5.0992500000000005</v>
+        <v>5.2980001422044172</v>
       </c>
       <c r="R24">
-        <v>5.3780300000000008</v>
+        <v>7.9470002133066266</v>
       </c>
       <c r="S24">
-        <v>0.50898031527096732</v>
+        <v>4.8363903125848955</v>
       </c>
       <c r="T24">
         <v>3.96</v>
@@ -2233,19 +2233,19 @@
         <v>11.142600000000002</v>
       </c>
       <c r="G25">
-        <v>9003.7900000000009</v>
+        <v>905.77200000000005</v>
       </c>
       <c r="H25">
-        <v>1844.81</v>
+        <v>3156.07</v>
       </c>
       <c r="I25">
-        <v>13.422503634580549</v>
+        <v>499.56191933510854</v>
       </c>
       <c r="J25">
         <v>459.5</v>
       </c>
       <c r="K25">
-        <v>-134.24096330090651</v>
+        <v>-4.9956191933510858</v>
       </c>
       <c r="L25">
         <v>-60</v>
@@ -2257,19 +2257,19 @@
         <v>0</v>
       </c>
       <c r="O25">
-        <v>13.422503634580549</v>
+        <v>499.56191933510854</v>
       </c>
       <c r="P25">
-        <v>0.898899</v>
+        <v>0.49306750000000354</v>
       </c>
       <c r="Q25">
-        <v>1.3580794999999999</v>
+        <v>0.98613500000000709</v>
       </c>
       <c r="R25">
-        <v>1.8172600000000001</v>
+        <v>1.4792025000000106</v>
       </c>
       <c r="S25">
-        <v>0.83834505938833637</v>
+        <v>0.90021397374226808</v>
       </c>
       <c r="T25">
         <v>11.14</v>
@@ -2301,19 +2301,19 @@
         <v>5.6056000000000008</v>
       </c>
       <c r="G26">
-        <v>681.51</v>
+        <v>1024.46</v>
       </c>
       <c r="H26">
-        <v>5537.94</v>
+        <v>7.0429000000000004</v>
       </c>
       <c r="I26">
-        <v>51.196775542545232</v>
+        <v>56.485673125353834</v>
       </c>
       <c r="J26">
         <v>459.5</v>
       </c>
       <c r="K26">
-        <v>-512.02850480333166</v>
+        <v>-0.5648567312535383</v>
       </c>
       <c r="L26">
         <v>-60</v>
@@ -2325,19 +2325,19 @@
         <v>0</v>
       </c>
       <c r="O26">
-        <v>51.196775542545232</v>
+        <v>56.485673125353834</v>
       </c>
       <c r="P26">
-        <v>4.9784199999999998</v>
+        <v>2.6022550000000346</v>
       </c>
       <c r="Q26">
-        <v>5.2467050000000004</v>
+        <v>5.2045100000000692</v>
       </c>
       <c r="R26">
-        <v>5.5149900000000001</v>
+        <v>7.8067650000001043</v>
       </c>
       <c r="S26">
-        <v>0.48981915446757834</v>
+        <v>4.7510458796020831</v>
       </c>
       <c r="T26">
         <v>5.61</v>
@@ -2369,19 +2369,19 @@
         <v>2.9204000000000003</v>
       </c>
       <c r="G27">
-        <v>7146.8</v>
+        <v>97.383099999999999</v>
       </c>
       <c r="H27">
-        <v>122.63</v>
+        <v>743.61599999999999</v>
       </c>
       <c r="I27">
-        <v>2.9701034868752449</v>
+        <v>252.17079472721653</v>
       </c>
       <c r="J27">
         <v>459.5</v>
       </c>
       <c r="K27">
-        <v>-29.704559152013509</v>
+        <v>-2.5217079472721653</v>
       </c>
       <c r="L27">
         <v>-60</v>
@@ -2393,19 +2393,19 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <v>2.9701034868752449</v>
+        <v>252.17079472721653</v>
       </c>
       <c r="P27">
-        <v>2.0953599999999999</v>
+        <v>1.0982749694460421</v>
       </c>
       <c r="Q27">
-        <v>2.299105</v>
+        <v>2.1965499388920842</v>
       </c>
       <c r="R27">
-        <v>2.50285</v>
+        <v>3.2948249083381267</v>
       </c>
       <c r="S27">
-        <v>0.37198577492963347</v>
+        <v>2.0051665836963144</v>
       </c>
       <c r="T27">
         <v>2.92</v>
@@ -2437,19 +2437,19 @@
         <v>2.9988000000000006</v>
       </c>
       <c r="G28">
-        <v>7912.13</v>
+        <v>183.77199999999999</v>
       </c>
       <c r="H28">
-        <v>726.36</v>
+        <v>3026.63</v>
       </c>
       <c r="I28">
-        <v>3.2754100349716193</v>
+        <v>524.08451777202185</v>
       </c>
       <c r="J28">
         <v>459.5</v>
       </c>
       <c r="K28">
-        <v>-32.75798690545755</v>
+        <v>-5.2408451777202183</v>
       </c>
       <c r="L28">
         <v>-60</v>
@@ -2461,19 +2461,19 @@
         <v>0</v>
       </c>
       <c r="O28">
-        <v>3.2754100349716193</v>
+        <v>524.08451777202185</v>
       </c>
       <c r="P28">
-        <v>1.75936</v>
+        <v>0.89187500000000375</v>
       </c>
       <c r="Q28">
-        <v>1.8021200000000002</v>
+        <v>1.7837500000000075</v>
       </c>
       <c r="R28">
-        <v>1.8448800000000001</v>
+        <v>2.6756250000000112</v>
       </c>
       <c r="S28">
-        <v>7.8068721863069707E-2</v>
+        <v>1.6283335199164071</v>
       </c>
       <c r="T28">
         <v>3</v>
@@ -2505,19 +2505,19 @@
         <v>10.221400000000001</v>
       </c>
       <c r="G29">
-        <v>48.14</v>
+        <v>97.020099999999999</v>
       </c>
       <c r="H29">
-        <v>9685.31</v>
+        <v>1618.85</v>
       </c>
       <c r="I29">
-        <v>2066.3867677606977</v>
+        <v>1807.4803491235318</v>
       </c>
       <c r="J29">
         <v>459.5</v>
       </c>
       <c r="K29">
-        <v>-20666.31962324748</v>
+        <v>-18.074803491235318</v>
       </c>
       <c r="L29">
         <v>-60</v>
@@ -2529,19 +2529,19 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <v>2066.3867677606977</v>
+        <v>1807.4803491235318</v>
       </c>
       <c r="P29">
-        <v>1.9027599999999998</v>
+        <v>1.7937150000000086</v>
       </c>
       <c r="Q29">
-        <v>3.7263600000000001</v>
+        <v>3.5874300000000172</v>
       </c>
       <c r="R29">
-        <v>5.5499600000000004</v>
+        <v>5.3811450000000258</v>
       </c>
       <c r="S29">
-        <v>3.3294228528880696</v>
+        <v>3.2748605574512792</v>
       </c>
       <c r="T29">
         <v>10.220000000000001</v>
@@ -2573,19 +2573,19 @@
         <v>1.3916000000000002</v>
       </c>
       <c r="G30">
-        <v>47.45</v>
+        <v>2</v>
       </c>
       <c r="H30">
-        <v>373.96</v>
+        <v>1044.54</v>
       </c>
       <c r="I30">
-        <v>40.320366701791357</v>
+        <v>23756.457999999999</v>
       </c>
       <c r="J30">
         <v>459.5</v>
       </c>
       <c r="K30">
-        <v>-403.25151060116735</v>
+        <v>-237.56457999999998</v>
       </c>
       <c r="L30">
         <v>-60</v>
@@ -2597,19 +2597,19 @@
         <v>0</v>
       </c>
       <c r="O30">
-        <v>40.320366701791357</v>
+        <v>23756.457999999999</v>
       </c>
       <c r="P30">
-        <v>2.3384100000000001</v>
+        <v>2.3406300000000346</v>
       </c>
       <c r="Q30">
-        <v>4.7607200000000001</v>
+        <v>4.6812600000000693</v>
       </c>
       <c r="R30">
-        <v>7.1830299999999996</v>
+        <v>7.0218900000001039</v>
       </c>
       <c r="S30">
-        <v>4.422512760901129</v>
+        <v>4.2733861659111199</v>
       </c>
       <c r="T30">
         <v>4.54</v>
@@ -2641,19 +2641,19 @@
         <v>4.5374000000000008</v>
       </c>
       <c r="G31">
-        <v>65.55</v>
+        <v>2.9293</v>
       </c>
       <c r="H31">
-        <v>361.16</v>
+        <v>1443.09</v>
       </c>
       <c r="I31">
-        <v>29.553980167810838</v>
+        <v>22411.250544498685</v>
       </c>
       <c r="J31">
         <v>459.5</v>
       </c>
       <c r="K31">
-        <v>-295.57487001766737</v>
+        <v>-224.11250544498685</v>
       </c>
       <c r="L31">
         <v>-60</v>
@@ -2665,19 +2665,19 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <v>29.553980167810838</v>
+        <v>22411.250544498685</v>
       </c>
       <c r="P31">
-        <v>1.76142</v>
+        <v>1.9726299999999881</v>
       </c>
       <c r="Q31">
-        <v>4.2218200000000001</v>
+        <v>3.9452599999999762</v>
       </c>
       <c r="R31">
-        <v>6.68222</v>
+        <v>5.9178899999999643</v>
       </c>
       <c r="S31">
-        <v>4.4920552682857027</v>
+        <v>3.6015131620380307</v>
       </c>
       <c r="T31">
         <v>4.54</v>
@@ -2709,19 +2709,19 @@
         <v>1.4210000000000003</v>
       </c>
       <c r="G32">
-        <v>151.31</v>
+        <v>470.85500000000002</v>
       </c>
       <c r="H32">
-        <v>9608.56</v>
+        <v>610.11400000000003</v>
       </c>
       <c r="I32">
-        <v>91.593519265084907</v>
+        <v>32.59975958628452</v>
       </c>
       <c r="J32">
         <v>459.5</v>
       </c>
       <c r="K32">
-        <v>-916.0438762398868</v>
+        <v>-0.32599759586284521</v>
       </c>
       <c r="L32">
         <v>-60</v>
@@ -2733,19 +2733,19 @@
         <v>0</v>
       </c>
       <c r="O32">
-        <v>91.593519265084907</v>
+        <v>32.59975958628452</v>
       </c>
       <c r="P32">
-        <v>3.8263199999999999</v>
+        <v>2.1487700000000256</v>
       </c>
       <c r="Q32">
-        <v>4.2885099999999996</v>
+        <v>4.2975400000000512</v>
       </c>
       <c r="R32">
-        <v>4.7507000000000001</v>
+        <v>6.4463100000000768</v>
       </c>
       <c r="S32">
-        <v>0.84383962951104263</v>
+        <v>3.9230993329679658</v>
       </c>
       <c r="T32">
         <v>1.42</v>
@@ -2777,19 +2777,19 @@
         <v>3.8906000000000005</v>
       </c>
       <c r="G33">
-        <v>20.3</v>
+        <v>64.297899999999998</v>
       </c>
       <c r="H33">
-        <v>158.08000000000001</v>
+        <v>84.579899999999995</v>
       </c>
       <c r="I33">
-        <v>34.182177339901479</v>
+        <v>90.070537606982498</v>
       </c>
       <c r="J33">
         <v>459.5</v>
       </c>
       <c r="K33">
-        <v>-341.86233349261346</v>
+        <v>-0.90070537606982504</v>
       </c>
       <c r="L33">
         <v>-60</v>
@@ -2801,19 +2801,19 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>34.182177339901479</v>
+        <v>90.070537606982498</v>
       </c>
       <c r="P33">
-        <v>0.98814500000000005</v>
+        <v>1.2328849999999849</v>
       </c>
       <c r="Q33">
-        <v>2.4294074999999999</v>
+        <v>2.4657699999999698</v>
       </c>
       <c r="R33">
-        <v>3.8706699999999996</v>
+        <v>3.6986549999999547</v>
       </c>
       <c r="S33">
-        <v>2.6313732751209646</v>
+        <v>2.2509297510324946</v>
       </c>
       <c r="T33">
         <v>3.89</v>
@@ -2845,19 +2845,19 @@
         <v>8.6044000000000018</v>
       </c>
       <c r="G34">
-        <v>593.76</v>
+        <v>3586.4</v>
       </c>
       <c r="H34">
-        <v>81.900000000000006</v>
+        <v>3.0556999999999999</v>
       </c>
       <c r="I34">
-        <v>9.7862368633791412</v>
+        <v>86.073274091010489</v>
       </c>
       <c r="J34">
         <v>459.5</v>
       </c>
       <c r="K34">
-        <v>-97.873980845594389</v>
+        <v>-0.86073274091010488</v>
       </c>
       <c r="L34">
         <v>-60</v>
@@ -2869,19 +2869,19 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <v>9.7862368633791412</v>
+        <v>86.073274091010489</v>
       </c>
       <c r="P34">
-        <v>4.2087399999999997</v>
+        <v>2.2762900000000026</v>
       </c>
       <c r="Q34">
-        <v>4.5477850000000002</v>
+        <v>4.5525800000000052</v>
       </c>
       <c r="R34">
-        <v>4.8868300000000007</v>
+        <v>6.8288700000000073</v>
       </c>
       <c r="S34">
-        <v>0.61900864836446401</v>
+        <v>4.1559179347447861</v>
       </c>
       <c r="T34">
         <v>8.6</v>
@@ -2913,19 +2913,19 @@
         <v>3.5378000000000007</v>
       </c>
       <c r="G35">
-        <v>553.51</v>
+        <v>691.86</v>
       </c>
       <c r="H35">
-        <v>122.63</v>
+        <v>553.61599999999999</v>
       </c>
       <c r="I35">
-        <v>4.3242861014254492</v>
+        <v>63.726549301881896</v>
       </c>
       <c r="J35">
         <v>459.5</v>
       </c>
       <c r="K35">
-        <v>-43.24799215166793</v>
+        <v>-0.63726549301881896</v>
       </c>
       <c r="L35">
         <v>-60</v>
@@ -2937,19 +2937,19 @@
         <v>0</v>
       </c>
       <c r="O35">
-        <v>4.3242861014254492</v>
+        <v>63.726549301881896</v>
       </c>
       <c r="P35">
-        <v>4.0089100000000002</v>
+        <v>2.4548800000000441</v>
       </c>
       <c r="Q35">
-        <v>4.3204549999999999</v>
+        <v>4.9097600000000883</v>
       </c>
       <c r="R35">
-        <v>4.6319999999999997</v>
+        <v>7.364640000000132</v>
       </c>
       <c r="S35">
-        <v>0.56880074725982299</v>
+        <v>4.481977173227687</v>
       </c>
       <c r="T35">
         <v>3.54</v>
@@ -2981,19 +2981,19 @@
         <v>16.473800000000001</v>
       </c>
       <c r="G36">
-        <v>1371.48</v>
+        <v>853.93899999999996</v>
       </c>
       <c r="H36">
-        <v>1263.24</v>
+        <v>20.779599999999999</v>
       </c>
       <c r="I36">
-        <v>31.640153994225216</v>
+        <v>168.70778055575397</v>
       </c>
       <c r="J36">
         <v>459.5</v>
       </c>
       <c r="K36">
-        <v>-316.43908370649871</v>
+        <v>-1.6870778055575397</v>
       </c>
       <c r="L36">
         <v>-60</v>
@@ -3005,19 +3005,19 @@
         <v>0</v>
       </c>
       <c r="O36">
-        <v>31.640153994225216</v>
+        <v>168.70778055575397</v>
       </c>
       <c r="P36">
-        <v>3.9028199999999997</v>
+        <v>2.2448849999999969</v>
       </c>
       <c r="Q36">
-        <v>4.5866899999999999</v>
+        <v>4.4897699999999938</v>
       </c>
       <c r="R36">
-        <v>5.2705599999999997</v>
+        <v>6.7346549999999912</v>
       </c>
       <c r="S36">
-        <v>1.248570084670193</v>
+        <v>4.0985805116832763</v>
       </c>
       <c r="T36">
         <v>16.47</v>
@@ -3049,19 +3049,19 @@
         <v>2.5480000000000005</v>
       </c>
       <c r="G37">
-        <v>7396.8</v>
+        <v>1146.3</v>
       </c>
       <c r="H37">
-        <v>1391.24</v>
+        <v>2891.98</v>
       </c>
       <c r="I37">
-        <v>3.0296211875405583</v>
+        <v>89.833499084009404</v>
       </c>
       <c r="J37">
         <v>459.5</v>
       </c>
       <c r="K37">
-        <v>-30.299806781537903</v>
+        <v>-0.89833499084009405</v>
       </c>
       <c r="L37">
         <v>-60</v>
@@ -3073,19 +3073,19 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <v>3.0296211875405583</v>
+        <v>89.833499084009404</v>
       </c>
       <c r="P37">
-        <v>3.2658199999999997</v>
+        <v>1.8079300000000111</v>
       </c>
       <c r="Q37">
-        <v>3.5128949999999999</v>
+        <v>3.6158600000000223</v>
       </c>
       <c r="R37">
-        <v>3.75997</v>
+        <v>5.4237900000000332</v>
       </c>
       <c r="S37">
-        <v>0.45109516965196317</v>
+        <v>3.3008134779677367</v>
       </c>
       <c r="T37">
         <v>2.5499999999999998</v>
@@ -3117,19 +3117,19 @@
         <v>14.866600000000002</v>
       </c>
       <c r="G38">
-        <v>62.02</v>
+        <v>704.51900000000001</v>
       </c>
       <c r="H38">
-        <v>2077.0500000000002</v>
+        <v>318.55099999999999</v>
       </c>
       <c r="I38">
-        <v>512.86634795227349</v>
+        <v>215.93528208607572</v>
       </c>
       <c r="J38">
         <v>459.5</v>
       </c>
       <c r="K38">
-        <v>-5129.2720395588531</v>
+        <v>-2.1593528208607573</v>
       </c>
       <c r="L38">
         <v>-60</v>
@@ -3141,19 +3141,19 @@
         <v>0</v>
       </c>
       <c r="O38">
-        <v>512.86634795227349</v>
+        <v>215.93528208607572</v>
       </c>
       <c r="P38">
-        <v>3.8630800000000001</v>
+        <v>2.0798549999999811</v>
       </c>
       <c r="Q38">
-        <v>4.0290800000000004</v>
+        <v>4.1597099999999623</v>
       </c>
       <c r="R38">
-        <v>4.1950799999999999</v>
+        <v>6.2395649999999439</v>
       </c>
       <c r="S38">
-        <v>0.30307314848619221</v>
+        <v>3.7972783327996562</v>
       </c>
       <c r="T38">
         <v>14.87</v>
@@ -3185,19 +3185,19 @@
         <v>6.0760000000000005</v>
       </c>
       <c r="G39">
-        <v>9839.89</v>
+        <v>4192.0200000000004</v>
       </c>
       <c r="H39">
-        <v>4920.34</v>
+        <v>2751.18</v>
       </c>
       <c r="I39">
-        <v>9.1202440677690504</v>
+        <v>100.70242031288018</v>
       </c>
       <c r="J39">
         <v>459.5</v>
       </c>
       <c r="K39">
-        <v>-91.213262631756024</v>
+        <v>-1.0070242031288017</v>
       </c>
       <c r="L39">
         <v>-60</v>
@@ -3209,19 +3209,19 @@
         <v>0</v>
       </c>
       <c r="O39">
-        <v>9.1202440677690504</v>
+        <v>100.70242031288018</v>
       </c>
       <c r="P39">
-        <v>3.8449999999999998</v>
+        <v>2.0056350000000456</v>
       </c>
       <c r="Q39">
-        <v>4.0720700000000001</v>
+        <v>4.0112700000000912</v>
       </c>
       <c r="R39">
-        <v>4.2991399999999995</v>
+        <v>6.0169050000001363</v>
       </c>
       <c r="S39">
-        <v>0.41457120377566026</v>
+        <v>3.6617717720729956</v>
       </c>
       <c r="T39">
         <v>6.08</v>

</xml_diff>